<commit_message>
Add checkout test cases and standardize test types
</commit_message>
<xml_diff>
--- a/test-cases/cart-test-cases.xlsx
+++ b/test-cases/cart-test-cases.xlsx
@@ -28,12 +28,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="61">
   <si>
     <t>TC ID</t>
   </si>
   <si>
     <t>Title</t>
+  </si>
+  <si>
+    <t>Test Type</t>
   </si>
   <si>
     <t>Precondition</t>
@@ -1507,18 +1510,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G50"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="6"/>
+  <dimension ref="A1:H50"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
     <col min="2" max="2" width="39.125" customWidth="1"/>
-    <col min="3" max="3" width="47.25" customWidth="1"/>
-    <col min="4" max="4" width="39.75" customWidth="1"/>
-    <col min="5" max="5" width="54.3083333333333" customWidth="1"/>
-    <col min="6" max="6" width="48.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="17.7666666666667" customWidth="1"/>
+    <col min="4" max="4" width="47.25" customWidth="1"/>
+    <col min="5" max="5" width="39.75" customWidth="1"/>
+    <col min="6" max="6" width="54.3083333333333" customWidth="1"/>
+    <col min="7" max="7" width="48.3333333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:7">
+    <row r="1" ht="15.75" spans="1:8">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1540,17 +1544,18 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" ht="150" customHeight="1" spans="1:7">
+      <c r="H1" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" ht="150" customHeight="1" spans="1:8">
       <c r="A2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
+      <c r="C2" s="3"/>
       <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
@@ -1560,22 +1565,23 @@
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" ht="156" customHeight="1" spans="1:7">
+      <c r="H2" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" ht="156" customHeight="1" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="C3" s="3"/>
       <c r="D3" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>17</v>
@@ -1583,22 +1589,23 @@
       <c r="F3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" ht="138" customHeight="1" spans="1:7">
+      <c r="G3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" ht="138" customHeight="1" spans="1:8">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="C4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>22</v>
@@ -1606,20 +1613,21 @@
       <c r="F4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" ht="134" customHeight="1" spans="1:7">
+      <c r="G4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" ht="134" customHeight="1" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="3" t="s">
         <v>26</v>
       </c>
+      <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
         <v>27</v>
       </c>
@@ -1629,20 +1637,21 @@
       <c r="F5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" ht="166" customHeight="1" spans="1:7">
+      <c r="G5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" ht="166" customHeight="1" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="3" t="s">
         <v>32</v>
       </c>
+      <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
         <v>33</v>
       </c>
@@ -1652,20 +1661,21 @@
       <c r="F6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="112" customHeight="1" spans="1:7">
+      <c r="G6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="3" t="s">
         <v>38</v>
       </c>
+      <c r="C7" s="3"/>
       <c r="D7" s="3" t="s">
         <v>39</v>
       </c>
@@ -1675,11 +1685,14 @@
       <c r="F7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" ht="61" customHeight="1" spans="1:7">
+      <c r="G7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" ht="61" customHeight="1" spans="1:8">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1687,8 +1700,9 @@
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1696,8 +1710,9 @@
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9" s="8"/>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -1705,8 +1720,9 @@
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="H10" s="8"/>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -1714,8 +1730,9 @@
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="H11" s="8"/>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -1723,8 +1740,9 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="H12" s="8"/>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -1732,8 +1750,9 @@
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="H13" s="8"/>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -1741,8 +1760,9 @@
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="H14" s="8"/>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -1750,8 +1770,9 @@
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="H15" s="8"/>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -1759,8 +1780,9 @@
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="H16" s="8"/>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -1768,8 +1790,9 @@
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="H17" s="8"/>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -1777,8 +1800,9 @@
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="H18" s="8"/>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -1786,8 +1810,9 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="H19" s="8"/>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -1795,8 +1820,9 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="H20" s="8"/>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -1804,17 +1830,19 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="H21" s="8"/>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="9"/>
       <c r="G22" s="8"/>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="H22" s="8"/>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -1822,8 +1850,9 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="H23" s="8"/>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -1831,8 +1860,9 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="H24" s="8"/>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -1840,8 +1870,9 @@
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="H25" s="8"/>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -1849,8 +1880,9 @@
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="H26" s="8"/>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -1858,8 +1890,9 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="H27" s="8"/>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -1867,8 +1900,9 @@
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="H28" s="8"/>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -1876,8 +1910,9 @@
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="H29" s="8"/>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -1885,8 +1920,9 @@
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
       <c r="G30" s="8"/>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="H30" s="8"/>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" s="8"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -1894,8 +1930,9 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
-    </row>
-    <row r="32" spans="1:7">
+      <c r="H31" s="8"/>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -1903,8 +1940,9 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
       <c r="G32" s="8"/>
-    </row>
-    <row r="33" spans="1:7">
+      <c r="H32" s="8"/>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -1912,8 +1950,9 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
-    </row>
-    <row r="34" spans="1:7">
+      <c r="H33" s="8"/>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -1921,8 +1960,9 @@
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
-    </row>
-    <row r="35" spans="1:7">
+      <c r="H34" s="8"/>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -1930,8 +1970,9 @@
       <c r="E35" s="8"/>
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
-    </row>
-    <row r="36" spans="1:7">
+      <c r="H35" s="8"/>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -1939,8 +1980,9 @@
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
-    </row>
-    <row r="37" spans="1:7">
+      <c r="H36" s="8"/>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -1948,8 +1990,9 @@
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
-    </row>
-    <row r="38" spans="1:7">
+      <c r="H37" s="8"/>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -1957,8 +2000,9 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
-    </row>
-    <row r="39" spans="1:7">
+      <c r="H38" s="8"/>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" s="8"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -1966,8 +2010,9 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
       <c r="G39" s="8"/>
-    </row>
-    <row r="40" spans="1:7">
+      <c r="H39" s="8"/>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -1975,8 +2020,9 @@
       <c r="E40" s="8"/>
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
-    </row>
-    <row r="41" spans="1:7">
+      <c r="H40" s="8"/>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" s="8"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -1984,8 +2030,9 @@
       <c r="E41" s="8"/>
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
-    </row>
-    <row r="42" spans="1:7">
+      <c r="H41" s="8"/>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -1993,8 +2040,9 @@
       <c r="E42" s="8"/>
       <c r="F42" s="8"/>
       <c r="G42" s="8"/>
-    </row>
-    <row r="43" spans="1:7">
+      <c r="H42" s="8"/>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -2002,8 +2050,9 @@
       <c r="E43" s="8"/>
       <c r="F43" s="8"/>
       <c r="G43" s="8"/>
-    </row>
-    <row r="44" spans="1:7">
+      <c r="H43" s="8"/>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -2011,8 +2060,9 @@
       <c r="E44" s="8"/>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
-    </row>
-    <row r="45" spans="1:7">
+      <c r="H44" s="8"/>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45" s="8"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -2020,8 +2070,9 @@
       <c r="E45" s="8"/>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
-    </row>
-    <row r="46" spans="1:7">
+      <c r="H45" s="8"/>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -2029,8 +2080,9 @@
       <c r="E46" s="8"/>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
-    </row>
-    <row r="47" spans="1:7">
+      <c r="H46" s="8"/>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -2038,8 +2090,9 @@
       <c r="E47" s="8"/>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
-    </row>
-    <row r="48" spans="1:7">
+      <c r="H47" s="8"/>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -2047,8 +2100,9 @@
       <c r="E48" s="8"/>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
-    </row>
-    <row r="49" spans="1:7">
+      <c r="H48" s="8"/>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -2056,8 +2110,9 @@
       <c r="E49" s="8"/>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
-    </row>
-    <row r="50" spans="1:7">
+      <c r="H49" s="8"/>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -2065,6 +2120,7 @@
       <c r="E50" s="8"/>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2091,33 +2147,33 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" ht="121" customHeight="1" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="5">
@@ -2126,16 +2182,16 @@
     </row>
     <row r="3" ht="139" customHeight="1" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="5">
@@ -2144,16 +2200,16 @@
     </row>
     <row r="4" ht="84" customHeight="1" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="5">
@@ -2162,16 +2218,16 @@
     </row>
     <row r="5" ht="128" customHeight="1" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="5">
@@ -2180,16 +2236,16 @@
     </row>
     <row r="6" ht="156" customHeight="1" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="5">
@@ -2198,16 +2254,16 @@
     </row>
     <row r="7" ht="105" customHeight="1" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="5">

</xml_diff>

<commit_message>
Standardize test types and priorities across test cases
</commit_message>
<xml_diff>
--- a/test-cases/cart-test-cases.xlsx
+++ b/test-cases/cart-test-cases.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17580"/>
+    <workbookView windowWidth="25800" windowHeight="17580"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="63">
   <si>
     <t>TC ID</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>Verify Adding a Product to Cart</t>
+  </si>
+  <si>
+    <t>Positive</t>
   </si>
   <si>
     <t>1. ผู้ใช้เข้าสู่ระบบ (Login) สำเร็จและอยู่บนหน้า Products
@@ -137,6 +140,9 @@
    "Add to Cart" เป็น "Remove"
 2. ปุ่มของ Sauce Labs Bike Light ยังคงแสดง
    "Add to Cart" ไม่เปลี่ยนเป็น "Remove"</t>
+  </si>
+  <si>
+    <t>Medium</t>
   </si>
   <si>
     <t>TC-CART-004</t>
@@ -1520,6 +1526,7 @@
     <col min="5" max="5" width="39.75" customWidth="1"/>
     <col min="6" max="6" width="54.3083333333333" customWidth="1"/>
     <col min="7" max="7" width="48.3333333333333" customWidth="1"/>
+    <col min="8" max="8" width="12.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" spans="1:8">
@@ -1555,141 +1562,153 @@
       <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3"/>
+      <c r="C2" s="7" t="s">
+        <v>10</v>
+      </c>
       <c r="D2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" ht="156" customHeight="1" spans="1:8">
       <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>15</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" ht="138" customHeight="1" spans="1:8">
       <c r="A4" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>10</v>
+      </c>
       <c r="D4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" ht="134" customHeight="1" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>26</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" ht="166" customHeight="1" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>10</v>
+      </c>
       <c r="D6" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="112" customHeight="1" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="3"/>
+        <v>40</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>10</v>
+      </c>
       <c r="D7" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="61" customHeight="1" spans="1:8">
@@ -2147,19 +2166,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" ht="121" customHeight="1" spans="1:6">
@@ -2167,13 +2186,13 @@
         <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="5">
@@ -2182,16 +2201,16 @@
     </row>
     <row r="3" ht="139" customHeight="1" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="D3" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="5">
@@ -2200,16 +2219,16 @@
     </row>
     <row r="4" ht="84" customHeight="1" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="5">
@@ -2218,16 +2237,16 @@
     </row>
     <row r="5" ht="128" customHeight="1" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="5">
@@ -2236,16 +2255,16 @@
     </row>
     <row r="6" ht="156" customHeight="1" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="5">
@@ -2254,16 +2273,16 @@
     </row>
     <row r="7" ht="105" customHeight="1" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="5">

</xml_diff>

<commit_message>
Improve test execution evidence documentation
</commit_message>
<xml_diff>
--- a/test-cases/cart-test-cases.xlsx
+++ b/test-cases/cart-test-cases.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="165">
   <si>
     <t>SAUCEDEMO  /  SHOPPING CART</t>
   </si>
@@ -364,6 +364,9 @@
     <t>MANUAL QA TEST DOCUMENTATION   •   TEST EXECUTION RESULTS</t>
   </si>
   <si>
+    <t>Evidence screenshots are grouped by Test Case ID, not individually mapped to each Actual Result entry. One screenshot may support multiple observations.</t>
+  </si>
+  <si>
     <t>Actual Result</t>
   </si>
   <si>
@@ -382,84 +385,266 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>1. The Backpack "Add to cart" button changed to "Remove".
-2. The cart badge displayed 1.
-3. The cart contained exactly one Sauce Labs Backpack and no other items.</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1. The Backpack "Add to cart" button changed to "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Remove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>".</t>
+    </r>
   </si>
   <si>
     <t>PASS</t>
   </si>
   <si>
-    <t>1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png
-2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_AFTER.png
-3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_CART.png</t>
-  </si>
-  <si>
-    <t>1. All three selected products displayed "Remove" buttons.
-2. The cart badge displayed 3.
-3. The Shopping Cart contained Sauce Labs Backpack, Sauce Labs Bike Light, and Sauce Labs Bolt T-Shirt, with no other products.</t>
-  </si>
-  <si>
-    <t>1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png
-2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_PRODUCTS.png
-3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_CART.png</t>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png</t>
+  </si>
+  <si>
+    <t>2. The cart badge displayed 1.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_AFTER.png</t>
+  </si>
+  <si>
+    <t>3. The cart contained exactly one Sauce Labs Backpack and no other items.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_CART.png</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1. All three selected products displayed "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Remove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>" buttons.</t>
+    </r>
   </si>
   <si>
     <t>Shared setup evidence: TC-CART-001_BEFORE.png is reused to show the initial empty-cart state. TC-CART-002_PRODUCTS.png and TC-CART-002_CART.png document this test case.</t>
   </si>
   <si>
-    <t>1. The Backpack button changed from "Add to cart" to "Remove".
-2. The Bike Light button remained "Add to cart".</t>
-  </si>
-  <si>
-    <t>1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_BEFORE.png
-2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_AFTER.png</t>
-  </si>
-  <si>
-    <t>1. After adding Backpack, the cart badge displayed 1.
-2. After adding Bike Light, the cart badge displayed 2.
-3. After removing Backpack, the cart badge displayed 1.
-4. After removing Bike Light, the cart badge displayed no item count.</t>
-  </si>
-  <si>
-    <t>1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_01_EMPTY.png
-2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_02_BADGE_1.png
-3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_03_BADGE_2.png
-4. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_CART_2_ITEMS.png
-5. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_04_AFTER_REMOVE_1.png
-6. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_05_BADGE_CLEARED.png</t>
-  </si>
-  <si>
-    <t>1. The cart displayed Backpack ($29.99) and Bike Light ($9.99), each with quantity 1.
-2. Product names, descriptions, and prices matched the Products page.</t>
-  </si>
-  <si>
-    <t>1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_PRODUCTS.png
-2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_CART.png</t>
-  </si>
-  <si>
-    <t>1. Sauce Labs Backpack was removed from the cart.
-2. Sauce Labs Bike Light remained in the cart.
-3. The cart badge decreased from 2 to 1.</t>
-  </si>
-  <si>
-    <t>1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_CART_PAGE.png
-2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_BEFORE.png
-3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_AFTER.png</t>
-  </si>
-  <si>
-    <t>1. The Products page displayed Sauce Labs Backpack with the Remove button and a cart badge count of 1.
-2. The Shopping Cart contained one Sauce Labs Backpack priced at $29.99, and the Continue Shopping button was available.
-3. After clicking Continue Shopping, the application returned to the Products page.
-4. The cart badge still displayed 1, and the Backpack button remained Remove.
-5. After reopening the Shopping Cart, the Backpack remained in the cart with quantity 1 and price $29.99.</t>
-  </si>
-  <si>
-    <t>1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_01_PRODUCTS_BEFORE.png
-2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_02_CART_BEFORE.png
-3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_03_PRODUCTS_AFTER.png
-4. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_04_BADGE.png
-5. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_05_CART_AFTER.png</t>
+    <t>2. The cart badge displayed 3.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_PRODUCTS.png</t>
+  </si>
+  <si>
+    <t>3. The Shopping Cart contained Sauce Labs Backpack, Sauce Labs Bike Light, and Sauce Labs Bolt T-Shirt, with no other products.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_CART.png</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1. The Backpack button changed from "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">Add to cart" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>to</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> "Remove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>".</t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_BEFORE.png</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>2. The Bike Light button remained "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Add to cart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1D3348"/>
+        <rFont val="Aptos"/>
+        <charset val="134"/>
+      </rPr>
+      <t>".</t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_AFTER.png</t>
+  </si>
+  <si>
+    <t>1. After adding Backpack, the cart badge displayed 1.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_01_EMPTY.png</t>
+  </si>
+  <si>
+    <t>2. After adding Bike Light, the cart badge displayed 2.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_02_BADGE_1.png</t>
+  </si>
+  <si>
+    <t>3. After removing Backpack, the cart badge displayed 1.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_03_BADGE_2.png</t>
+  </si>
+  <si>
+    <t>4. After removing Bike Light, the cart badge displayed no item count.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_CART_2_ITEMS.png</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_04_AFTER_REMOVE_1.png</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_05_BADGE_CLEARED.png</t>
+  </si>
+  <si>
+    <t>1. The cart displayed Backpack ($29.99) and Bike Light ($9.99), each with quantity 1.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_PRODUCTS.png</t>
+  </si>
+  <si>
+    <t>2. Product names, descriptions, and prices matched the Products page.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_CART.png</t>
+  </si>
+  <si>
+    <t>1. Sauce Labs Backpack was removed from the cart.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_CART_PAGE.png</t>
+  </si>
+  <si>
+    <t>2. Sauce Labs Bike Light remained in the cart.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_BEFORE.png</t>
+  </si>
+  <si>
+    <t>3. The cart badge decreased from 2 to 1.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_AFTER.png</t>
+  </si>
+  <si>
+    <t>1. The Products page displayed Sauce Labs Backpack with the Remove button and a cart badge count of 1.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_01_PRODUCTS_BEFORE.png</t>
+  </si>
+  <si>
+    <t>2. The Shopping Cart contained one Sauce Labs Backpack priced at $29.99, and the Continue Shopping button was available.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_02_CART_BEFORE.png</t>
+  </si>
+  <si>
+    <t>3. After clicking Continue Shopping, the application returned to the Products page.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_03_PRODUCTS_AFTER.png</t>
+  </si>
+  <si>
+    <t>4. The cart badge still displayed 1, and the Backpack button remained Remove.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_04_BADGE.png</t>
+  </si>
+  <si>
+    <t>5. After reopening the Shopping Cart, the Backpack remained in the cart with quantity 1 and price $29.99.</t>
+  </si>
+  <si>
+    <t>https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_05_CART_AFTER.png</t>
   </si>
 </sst>
 </file>
@@ -473,7 +658,7 @@
     <numFmt numFmtId="179" formatCode="_-&quot;฿&quot;* #,##0_-;\-&quot;฿&quot;* #,##0_-;_-&quot;฿&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="180" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -498,6 +683,12 @@
       <sz val="10"/>
       <color rgb="FF17365D"/>
       <name val="Aptos"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF002060"/>
+      <name val="Carlito"/>
       <charset val="134"/>
     </font>
     <font>
@@ -650,6 +841,17 @@
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Aptos"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="40">
     <fill>
@@ -887,7 +1089,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -961,16 +1163,38 @@
     </border>
     <border>
       <left style="hair">
-        <color rgb="FF303944"/>
+        <color auto="1"/>
       </left>
       <right style="hair">
-        <color rgb="FF303944"/>
+        <color auto="1"/>
       </right>
       <top style="hair">
-        <color rgb="FF303944"/>
+        <color auto="1"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top/>
       <bottom style="hair">
-        <color rgb="FF303944"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1002,6 +1226,21 @@
       <top/>
       <bottom style="hair">
         <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="FF303944"/>
+      </left>
+      <right style="hair">
+        <color rgb="FF303944"/>
+      </right>
+      <top style="hair">
+        <color rgb="FF303944"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="FF303944"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1106,31 +1345,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1139,119 +1375,122 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1274,130 +1513,217 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="5" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1455,7 +1781,17 @@
   <dxfs count="22">
     <dxf>
       <font>
-        <color theme="9"/>
+        <color theme="5"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0070C0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
       </font>
     </dxf>
     <dxf>
@@ -1465,17 +1801,7 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF0070C0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5"/>
+        <color theme="9"/>
       </font>
     </dxf>
     <dxf>
@@ -1912,24 +2238,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="56"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:7">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="34"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="58"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:7">
       <c r="A3" s="5" t="s">
@@ -1937,19 +2263,19 @@
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="35"/>
-      <c r="F3" s="36"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="60"/>
     </row>
     <row r="4" ht="11" customHeight="1" spans="1:7">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="37"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="63"/>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:7">
       <c r="A5" s="10" t="s">
@@ -1970,168 +2296,168 @@
       <c r="F5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="46" t="s">
+      <c r="G5" s="72" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" ht="50" customHeight="1" spans="1:7">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="48" t="s">
+      <c r="D6" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="48" t="s">
+      <c r="F6" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="49" t="s">
+      <c r="G6" s="76" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1" spans="1:7">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="43" t="s">
+      <c r="F7" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="50" t="s">
+      <c r="G7" s="77" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" ht="50" customHeight="1" spans="1:7">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="48" t="s">
+      <c r="C8" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="48" t="s">
+      <c r="D8" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="48" t="s">
+      <c r="F8" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="49" t="s">
+      <c r="G8" s="76" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1" spans="1:7">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="43" t="s">
+      <c r="F9" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="50" t="s">
+      <c r="G9" s="77" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" ht="66" customHeight="1" spans="1:7">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="73" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="48" t="s">
+      <c r="D10" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="74" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="48" t="s">
+      <c r="F10" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="49" t="s">
+      <c r="G10" s="76" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="11" ht="66" customHeight="1" spans="1:7">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="43" t="s">
+      <c r="C11" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="43" t="s">
+      <c r="D11" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="43" t="s">
+      <c r="F11" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="50" t="s">
+      <c r="G11" s="77" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" ht="52" customHeight="1" spans="1:7">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="78" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="79" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="51" t="s">
+      <c r="C12" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="51" t="s">
+      <c r="D12" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="51" t="s">
+      <c r="F12" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="49" t="s">
+      <c r="G12" s="76" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2166,40 +2492,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:5">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="31"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="56"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:5">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="34"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="58"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:5">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="6"/>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="35"/>
-      <c r="E3" s="36"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
     </row>
     <row r="4" ht="11" customHeight="1" spans="1:5">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="37"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="63"/>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5">
       <c r="A5" s="10" t="s">
@@ -2219,496 +2545,496 @@
       </c>
     </row>
     <row r="6" ht="29" customHeight="1" spans="1:5">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="39">
+      <c r="B6" s="65">
         <v>1</v>
       </c>
-      <c r="C6" s="40" t="s">
+      <c r="C6" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="40" t="s">
+      <c r="E6" s="12" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="7" ht="29" customHeight="1" spans="1:5">
-      <c r="A7" s="41"/>
-      <c r="B7" s="39">
+      <c r="A7" s="66"/>
+      <c r="B7" s="65">
         <v>2</v>
       </c>
-      <c r="C7" s="40" t="s">
+      <c r="C7" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="12" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="8" ht="29" customHeight="1" spans="1:5">
-      <c r="A8" s="41"/>
-      <c r="B8" s="39">
+      <c r="A8" s="66"/>
+      <c r="B8" s="65">
         <v>3</v>
       </c>
-      <c r="C8" s="40" t="s">
+      <c r="C8" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="40" t="s">
+      <c r="E8" s="12" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="9" ht="29" customHeight="1" spans="1:5">
-      <c r="A9" s="41"/>
-      <c r="B9" s="39">
+      <c r="A9" s="66"/>
+      <c r="B9" s="65">
         <v>4</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="C9" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="40" t="s">
+      <c r="D9" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="40" t="s">
+      <c r="E9" s="12" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5">
-      <c r="A10" s="41"/>
-      <c r="B10" s="39">
+      <c r="A10" s="66"/>
+      <c r="B10" s="65">
         <v>5</v>
       </c>
-      <c r="C10" s="40" t="s">
+      <c r="C10" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="40" t="s">
+      <c r="E10" s="12" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11" ht="29" customHeight="1" spans="1:5">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="43">
+      <c r="B11" s="68">
         <v>1</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="27" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="12" ht="29" customHeight="1" spans="1:5">
-      <c r="A12" s="21"/>
-      <c r="B12" s="43">
+      <c r="A12" s="69"/>
+      <c r="B12" s="68">
         <v>2</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="27" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="13" ht="29" customHeight="1" spans="1:5">
-      <c r="A13" s="21"/>
-      <c r="B13" s="43">
+      <c r="A13" s="69"/>
+      <c r="B13" s="68">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="27" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" ht="29" customHeight="1" spans="1:5">
-      <c r="A14" s="21"/>
-      <c r="B14" s="43">
+      <c r="A14" s="69"/>
+      <c r="B14" s="68">
         <v>4</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="27" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="15" ht="29" customHeight="1" spans="1:5">
-      <c r="A15" s="21"/>
-      <c r="B15" s="43">
+      <c r="A15" s="69"/>
+      <c r="B15" s="68">
         <v>5</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="27" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="16" ht="29" customHeight="1" spans="1:5">
-      <c r="A16" s="21"/>
-      <c r="B16" s="43">
+      <c r="A16" s="69"/>
+      <c r="B16" s="68">
         <v>6</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="27" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5">
-      <c r="A17" s="21"/>
-      <c r="B17" s="43">
+      <c r="A17" s="69"/>
+      <c r="B17" s="68">
         <v>7</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="27" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="18" ht="29" customHeight="1" spans="1:5">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="39">
+      <c r="B18" s="65">
         <v>1</v>
       </c>
-      <c r="C18" s="40" t="s">
+      <c r="C18" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="40" t="s">
+      <c r="D18" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="40" t="s">
+      <c r="E18" s="12" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" ht="29" customHeight="1" spans="1:5">
-      <c r="A19" s="41"/>
-      <c r="B19" s="39">
+      <c r="A19" s="66"/>
+      <c r="B19" s="65">
         <v>2</v>
       </c>
-      <c r="C19" s="40" t="s">
+      <c r="C19" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="40" t="s">
+      <c r="E19" s="12" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5">
-      <c r="A20" s="41"/>
-      <c r="B20" s="39">
+      <c r="A20" s="66"/>
+      <c r="B20" s="65">
         <v>3</v>
       </c>
-      <c r="C20" s="40" t="s">
+      <c r="C20" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="40" t="s">
+      <c r="E20" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="21" ht="29" customHeight="1" spans="1:5">
-      <c r="A21" s="41"/>
-      <c r="B21" s="39">
+      <c r="A21" s="66"/>
+      <c r="B21" s="65">
         <v>4</v>
       </c>
-      <c r="C21" s="40" t="s">
+      <c r="C21" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="D21" s="40" t="s">
+      <c r="D21" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E21" s="40" t="s">
+      <c r="E21" s="12" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="22" ht="29" customHeight="1" spans="1:5">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="43">
+      <c r="B22" s="68">
         <v>1</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="27" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="23" ht="29" customHeight="1" spans="1:5">
-      <c r="A23" s="21"/>
-      <c r="B23" s="43">
+      <c r="A23" s="69"/>
+      <c r="B23" s="68">
         <v>2</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="27" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="24" ht="29" customHeight="1" spans="1:5">
-      <c r="A24" s="21"/>
-      <c r="B24" s="43">
+      <c r="A24" s="69"/>
+      <c r="B24" s="68">
         <v>3</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="27" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="25" ht="29" customHeight="1" spans="1:5">
-      <c r="A25" s="21"/>
-      <c r="B25" s="43">
+      <c r="A25" s="69"/>
+      <c r="B25" s="68">
         <v>4</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="18" t="s">
+      <c r="E25" s="27" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="26" ht="42" customHeight="1" spans="1:5">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="39">
+      <c r="B26" s="65">
         <v>1</v>
       </c>
-      <c r="C26" s="40" t="s">
+      <c r="C26" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="D26" s="40" t="s">
+      <c r="D26" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="E26" s="40" t="s">
+      <c r="E26" s="12" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" ht="29" customHeight="1" spans="1:5">
-      <c r="A27" s="41"/>
-      <c r="B27" s="39">
+      <c r="A27" s="66"/>
+      <c r="B27" s="65">
         <v>2</v>
       </c>
-      <c r="C27" s="40" t="s">
+      <c r="C27" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="D27" s="40" t="s">
+      <c r="D27" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="E27" s="40" t="s">
+      <c r="E27" s="12" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="28" ht="42" customHeight="1" spans="1:5">
-      <c r="A28" s="41"/>
-      <c r="B28" s="39">
+      <c r="A28" s="66"/>
+      <c r="B28" s="65">
         <v>3</v>
       </c>
-      <c r="C28" s="40" t="s">
+      <c r="C28" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="40" t="s">
+      <c r="D28" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E28" s="40" t="s">
+      <c r="E28" s="12" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1" spans="1:5">
-      <c r="A29" s="41"/>
-      <c r="B29" s="39">
+      <c r="A29" s="66"/>
+      <c r="B29" s="65">
         <v>4</v>
       </c>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D29" s="40" t="s">
+      <c r="D29" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="E29" s="40" t="s">
+      <c r="E29" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="30" ht="42" customHeight="1" spans="1:5">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="43">
+      <c r="B30" s="68">
         <v>1</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="27" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="31" ht="29" customHeight="1" spans="1:5">
-      <c r="A31" s="21"/>
-      <c r="B31" s="43">
+      <c r="A31" s="69"/>
+      <c r="B31" s="68">
         <v>2</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="18" t="s">
+      <c r="E31" s="27" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="32" ht="29" customHeight="1" spans="1:5">
-      <c r="A32" s="21"/>
-      <c r="B32" s="43">
+      <c r="A32" s="69"/>
+      <c r="B32" s="68">
         <v>3</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="E32" s="18" t="s">
+      <c r="E32" s="27" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="33" ht="42" customHeight="1" spans="1:5">
-      <c r="A33" s="21"/>
-      <c r="B33" s="43">
+      <c r="A33" s="69"/>
+      <c r="B33" s="68">
         <v>4</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="D33" s="18" t="s">
+      <c r="D33" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E33" s="18" t="s">
+      <c r="E33" s="27" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="34" ht="37" customHeight="1" spans="1:5">
-      <c r="A34" s="44" t="s">
+      <c r="A34" s="70" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="39">
+      <c r="B34" s="65">
         <v>1</v>
       </c>
-      <c r="C34" s="40" t="s">
+      <c r="C34" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="D34" s="40" t="s">
+      <c r="D34" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E34" s="40" t="s">
+      <c r="E34" s="12" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="35" ht="33" customHeight="1" spans="1:5">
-      <c r="A35" s="45"/>
-      <c r="B35" s="39">
+      <c r="A35" s="71"/>
+      <c r="B35" s="65">
         <v>2</v>
       </c>
-      <c r="C35" s="40" t="s">
+      <c r="C35" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="D35" s="40" t="s">
+      <c r="D35" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="E35" s="40" t="s">
+      <c r="E35" s="12" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="36" ht="34" customHeight="1" spans="1:5">
-      <c r="A36" s="45"/>
-      <c r="B36" s="39">
+      <c r="A36" s="71"/>
+      <c r="B36" s="65">
         <v>3</v>
       </c>
-      <c r="C36" s="40" t="s">
+      <c r="C36" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="D36" s="40" t="s">
+      <c r="D36" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="E36" s="40" t="s">
+      <c r="E36" s="12" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="37" ht="36" customHeight="1" spans="1:5">
-      <c r="A37" s="45"/>
-      <c r="B37" s="39">
+      <c r="A37" s="71"/>
+      <c r="B37" s="65">
         <v>4</v>
       </c>
-      <c r="C37" s="40" t="s">
+      <c r="C37" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="D37" s="40" t="s">
+      <c r="D37" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E37" s="40" t="s">
+      <c r="E37" s="12" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2734,13 +3060,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="66.875" customWidth="1"/>
+    <col min="4" max="4" width="110" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="52" customWidth="1"/>
@@ -2782,8 +3108,10 @@
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
     </row>
-    <row r="4" ht="11" customHeight="1" spans="1:7">
-      <c r="A4" s="8"/>
+    <row r="4" customFormat="1" ht="23" customHeight="1" spans="1:7">
+      <c r="A4" s="8" t="s">
+        <v>111</v>
+      </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
@@ -2796,36 +3124,36 @@
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" ht="144" customHeight="1" spans="1:7">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" ht="39" customHeight="1" spans="1:7">
       <c r="A6" s="11" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="16">
@@ -2833,175 +3161,447 @@
       </c>
       <c r="G6" s="15"/>
     </row>
-    <row r="7" ht="144" customHeight="1" spans="1:7">
-      <c r="A7" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D7" s="20" t="s">
+    <row r="7" ht="38" customHeight="1" spans="1:7">
+      <c r="A7" s="17"/>
+      <c r="B7" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="E7" s="21"/>
-      <c r="F7" s="22">
-        <v>46306</v>
-      </c>
-      <c r="G7" s="23" t="s">
+      <c r="C7" s="18"/>
+      <c r="D7" s="19" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="8" ht="131" customHeight="1" spans="1:7">
-      <c r="A8" s="11" t="s">
-        <v>20</v>
-      </c>
+      <c r="E7" s="20"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="20"/>
+    </row>
+    <row r="8" ht="40" customHeight="1" spans="1:7">
+      <c r="A8" s="22"/>
       <c r="B8" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D8" s="24" t="s">
+      <c r="C8" s="23"/>
+      <c r="D8" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="16">
+      <c r="E8" s="24"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="24"/>
+    </row>
+    <row r="9" ht="39" customHeight="1" spans="1:7">
+      <c r="A9" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="E9" s="30"/>
+      <c r="F9" s="31">
         <v>46306</v>
       </c>
-      <c r="G8" s="15"/>
-    </row>
-    <row r="9" ht="272" customHeight="1" spans="1:7">
-      <c r="A9" s="17" t="s">
+      <c r="G9" s="32" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1" spans="1:7">
+      <c r="A10" s="33"/>
+      <c r="B10" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="34"/>
+      <c r="D10" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="E10" s="36"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="38"/>
+    </row>
+    <row r="11" ht="39" customHeight="1" spans="1:7">
+      <c r="A11" s="39"/>
+      <c r="B11" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" s="40"/>
+      <c r="D11" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="43"/>
+    </row>
+    <row r="12" ht="39" customHeight="1" spans="1:7">
+      <c r="A12" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="E12" s="15"/>
+      <c r="F12" s="16">
+        <v>46306</v>
+      </c>
+      <c r="G12" s="15"/>
+    </row>
+    <row r="13" ht="39" customHeight="1" spans="1:7">
+      <c r="A13" s="22"/>
+      <c r="B13" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C13" s="23"/>
+      <c r="D13" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="E13" s="24"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" ht="40" customHeight="1" spans="1:7">
+      <c r="A14" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="18" t="s">
-        <v>125</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="E9" s="21"/>
-      <c r="F9" s="22">
+      <c r="B14" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" s="30"/>
+      <c r="F14" s="31">
         <v>46306</v>
       </c>
-      <c r="G9" s="21"/>
-    </row>
-    <row r="10" ht="123" customHeight="1" spans="1:7">
-      <c r="A10" s="11" t="s">
+      <c r="G14" s="30"/>
+    </row>
+    <row r="15" ht="41" customHeight="1" spans="1:7">
+      <c r="A15" s="33"/>
+      <c r="B15" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="C15" s="34"/>
+      <c r="D15" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="E15" s="36"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="36"/>
+    </row>
+    <row r="16" ht="43" customHeight="1" spans="1:7">
+      <c r="A16" s="33"/>
+      <c r="B16" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="C16" s="34"/>
+      <c r="D16" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E16" s="36"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="36"/>
+    </row>
+    <row r="17" ht="40" customHeight="1" spans="1:7">
+      <c r="A17" s="33"/>
+      <c r="B17" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="C17" s="34"/>
+      <c r="D17" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="E17" s="36"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="36"/>
+    </row>
+    <row r="18" ht="46" customHeight="1" spans="1:7">
+      <c r="A18" s="33"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="E18" s="36"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="36"/>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="1:7">
+      <c r="A19" s="39"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="E19" s="41"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="41"/>
+    </row>
+    <row r="20" ht="45" customHeight="1" spans="1:7">
+      <c r="A20" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16">
+      <c r="B20" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="E20" s="15"/>
+      <c r="F20" s="16">
         <v>46306</v>
       </c>
-      <c r="G10" s="15"/>
-    </row>
-    <row r="11" ht="137" customHeight="1" spans="1:7">
-      <c r="A11" s="17" t="s">
+      <c r="G20" s="15"/>
+    </row>
+    <row r="21" ht="40" customHeight="1" spans="1:7">
+      <c r="A21" s="22"/>
+      <c r="B21" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="C21" s="23"/>
+      <c r="D21" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="E21" s="24"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="24"/>
+    </row>
+    <row r="22" ht="39" customHeight="1" spans="1:7">
+      <c r="A22" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>130</v>
-      </c>
-      <c r="E11" s="21"/>
-      <c r="F11" s="22">
+      <c r="B22" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E22" s="30"/>
+      <c r="F22" s="31">
         <v>46306</v>
       </c>
-      <c r="G11" s="21"/>
-    </row>
-    <row r="12" ht="198" customHeight="1" spans="1:7">
-      <c r="A12" s="25" t="s">
+      <c r="G22" s="30"/>
+    </row>
+    <row r="23" ht="40" customHeight="1" spans="1:7">
+      <c r="A23" s="33"/>
+      <c r="B23" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" s="34"/>
+      <c r="D23" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="E23" s="36"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="36"/>
+    </row>
+    <row r="24" ht="42" customHeight="1" spans="1:7">
+      <c r="A24" s="39"/>
+      <c r="B24" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="C24" s="40"/>
+      <c r="D24" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="E24" s="41"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="41"/>
+    </row>
+    <row r="25" ht="54" customHeight="1" spans="1:7">
+      <c r="A25" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D12" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="E12" s="26"/>
-      <c r="F12" s="28">
+      <c r="B25" s="45" t="s">
+        <v>155</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D25" s="46" t="s">
+        <v>156</v>
+      </c>
+      <c r="E25" s="47"/>
+      <c r="F25" s="48">
         <v>46311</v>
       </c>
-      <c r="G12" s="26"/>
+      <c r="G25" s="47"/>
+    </row>
+    <row r="26" ht="42" customHeight="1" spans="1:7">
+      <c r="A26" s="49"/>
+      <c r="B26" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="C26" s="18"/>
+      <c r="D26" s="50" t="s">
+        <v>158</v>
+      </c>
+      <c r="E26" s="51"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="51"/>
+    </row>
+    <row r="27" ht="41" customHeight="1" spans="1:7">
+      <c r="A27" s="49"/>
+      <c r="B27" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="C27" s="18"/>
+      <c r="D27" s="50" t="s">
+        <v>160</v>
+      </c>
+      <c r="E27" s="51"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="51"/>
+    </row>
+    <row r="28" ht="42" customHeight="1" spans="1:7">
+      <c r="A28" s="49"/>
+      <c r="B28" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="C28" s="18"/>
+      <c r="D28" s="50" t="s">
+        <v>162</v>
+      </c>
+      <c r="E28" s="51"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="51"/>
+    </row>
+    <row r="29" ht="47" customHeight="1" spans="1:7">
+      <c r="A29" s="53"/>
+      <c r="B29" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="C29" s="23"/>
+      <c r="D29" s="46" t="s">
+        <v>164</v>
+      </c>
+      <c r="E29" s="54"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="54"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="41">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="E3:G3"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A25:A29"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="C9:C11"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="C14:C19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="C25:C29"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E19"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="E25:E29"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="F14:F19"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="F25:F29"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="G14:G19"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="G22:G24"/>
+    <mergeCell ref="G25:G29"/>
   </mergeCells>
-  <conditionalFormatting sqref="C12">
-    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
-      <formula>"PASS"</formula>
+  <conditionalFormatting sqref="C25">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"NEEDS CLARIFICATION"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
-      <formula>"FAIL"</formula>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"NOT RUN"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"BLOCKED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
-      <formula>"NOT RUN"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"FAIL"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"PASS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6 C9 C12 C14 C20 C22">
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
       <formula>"NEEDS CLARIFICATION"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C11">
-    <cfRule type="cellIs" dxfId="0" priority="10" operator="equal">
-      <formula>"PASS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="9" operator="equal">
-      <formula>"FAIL"</formula>
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
+      <formula>"NOT RUN"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
       <formula>"BLOCKED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="7" operator="equal">
-      <formula>"NOT RUN"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
+      <formula>"FAIL"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
-      <formula>"NEEDS CLARIFICATION"</formula>
+    <cfRule type="cellIs" dxfId="4" priority="10" operator="equal">
+      <formula>"PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="C6:C12">
+    <dataValidation type="list" sqref="C6:C25">
       <formula1>"PASS,FAIL,BLOCKED,NOT RUN,NEEDS CLARIFICATION"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D11" r:id="rId1" display="1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_CART_PAGE.png&#10;&#10;2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_BEFORE.png&#10;&#10;3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_AFTER.png"/>
-    <hyperlink ref="D10" r:id="rId1" display="1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_PRODUCTS.png&#10;&#10;2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_CART.png"/>
-    <hyperlink ref="D9" r:id="rId1" display="1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_01_EMPTY.png&#10;&#10;2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_02_BADGE_1.png&#10;&#10;3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_03_BADGE_2.png&#10;&#10;4. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_CART_2_ITEMS.png&#10;&#10;5. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_04_AFTER_REMOVE_1.png&#10;&#10;6. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_05_BADGE_CLEARED.png"/>
-    <hyperlink ref="D8" r:id="rId1" display="1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_BEFORE.png&#10;&#10;2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_AFTER.png"/>
-    <hyperlink ref="D7" r:id="rId1" display="1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png&#10;&#10;2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_PRODUCTS.png&#10;&#10;3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_CART.png"/>
-    <hyperlink ref="D6" r:id="rId1" display="1. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png&#10;&#10;2. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_AFTER.png&#10;&#10;3. https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_CART.png"/>
+    <hyperlink ref="D22" r:id="rId1" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_CART_PAGE.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_CART_PAGE.png"/>
+    <hyperlink ref="D20" r:id="rId2" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_PRODUCTS.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_PRODUCTS.png"/>
+    <hyperlink ref="D14" r:id="rId3" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_01_EMPTY.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_01_EMPTY.png"/>
+    <hyperlink ref="D12" r:id="rId4" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_BEFORE.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_BEFORE.png"/>
+    <hyperlink ref="D9" r:id="rId5" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png"/>
+    <hyperlink ref="D6" r:id="rId5" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_BEFORE.png"/>
+    <hyperlink ref="D25" r:id="rId6" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_01_PRODUCTS_BEFORE.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_01_PRODUCTS_BEFORE.png"/>
+    <hyperlink ref="D7" r:id="rId7" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_AFTER.png"/>
+    <hyperlink ref="D8" r:id="rId8" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-001_CART.png"/>
+    <hyperlink ref="D10" r:id="rId9" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_PRODUCTS.png"/>
+    <hyperlink ref="D11" r:id="rId10" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-002_CART.png"/>
+    <hyperlink ref="D13" r:id="rId11" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-003_AFTER.png"/>
+    <hyperlink ref="D15" r:id="rId12" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_02_BADGE_1.png"/>
+    <hyperlink ref="D16" r:id="rId13" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_03_BADGE_2.png"/>
+    <hyperlink ref="D17" r:id="rId14" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_CART_2_ITEMS.png"/>
+    <hyperlink ref="D18" r:id="rId15" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_04_AFTER_REMOVE_1.png"/>
+    <hyperlink ref="D19" r:id="rId16" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-004_05_BADGE_CLEARED.png"/>
+    <hyperlink ref="D21" r:id="rId17" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-005_CART.png"/>
+    <hyperlink ref="D23" r:id="rId18" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_BEFORE.png"/>
+    <hyperlink ref="D24" r:id="rId19" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-006_AFTER.png"/>
+    <hyperlink ref="D26" r:id="rId20" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_02_CART_BEFORE.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_02_CART_BEFORE.png"/>
+    <hyperlink ref="D27" r:id="rId21" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_03_PRODUCTS_AFTER.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_03_PRODUCTS_AFTER.png"/>
+    <hyperlink ref="D28" r:id="rId22" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_04_BADGE.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_04_BADGE.png"/>
+    <hyperlink ref="D29" r:id="rId23" display="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_05_CART_AFTER.png" tooltip="https://github.com/kritsada-chaisongkram/saucedemo-manual-testing/blob/main/test-evidence/cart/TC-CART-007_05_CART_AFTER.png"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>